<commit_message>
Update raid chest averages and calendar navigation
</commit_message>
<xml_diff>
--- a/downloads/data/all-data.xlsx
+++ b/downloads/data/all-data.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research" sheetId="1" r:id="R93b03aea7e8445dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chest Data" sheetId="2" r:id="R51a124940b944860"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Army Data" sheetId="3" r:id="Rc1438f118d8f49e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research" sheetId="1" r:id="R1ed8a7d3adbe492e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chest Data" sheetId="2" r:id="R19d531c7c567429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Army Data" sheetId="3" r:id="Rf56fe232aaf848f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -27616,24 +27616,24 @@
         <x:v>561</x:v>
       </x:c>
       <x:c r="E46" t="n">
-        <x:v>288.36898395721926</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="F46" t="n">
-        <x:v>311.63101604278074</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="G46"/>
       <x:c r="H46"/>
       <x:c r="I46" t="n">
-        <x:v>47.89572192513369</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J46" t="n">
-        <x:v>68.3903743315508</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="K46" t="n">
-        <x:v>871.0695187165776</x:v>
+        <x:v>959</x:v>
       </x:c>
       <x:c r="L46" t="n">
-        <x:v>228074.86631016043</x:v>
+        <x:v>226282</x:v>
       </x:c>
       <x:c r="M46"/>
       <x:c r="N46"/>
@@ -27642,11 +27642,9 @@
       <x:c r="Q46"/>
       <x:c r="R46"/>
       <x:c r="S46" t="n">
-        <x:v>274.81283422459893</x:v>
-      </x:c>
-      <x:c r="T46" t="n">
-        <x:v>0.09759358288770054</x:v>
-      </x:c>
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="T46"/>
       <x:c r="U46"/>
     </x:row>
     <x:row r="47">
@@ -27663,24 +27661,24 @@
         <x:v>561</x:v>
       </x:c>
       <x:c r="E47" t="n">
-        <x:v>277.1436156092381</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="F47" t="n">
-        <x:v>309.7955933103265</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="G47"/>
       <x:c r="H47"/>
       <x:c r="I47" t="n">
-        <x:v>46.493230687549776</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J47" t="n">
-        <x:v>75.67560392885585</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="K47" t="n">
-        <x:v>848.6195911866207</x:v>
+        <x:v>959</x:v>
       </x:c>
       <x:c r="L47" t="n">
-        <x:v>225378.2851075126</x:v>
+        <x:v>226282</x:v>
       </x:c>
       <x:c r="M47"/>
       <x:c r="N47"/>
@@ -27689,11 +27687,9 @@
       <x:c r="Q47"/>
       <x:c r="R47"/>
       <x:c r="S47" t="n">
-        <x:v>259.9415980886647</x:v>
-      </x:c>
-      <x:c r="T47" t="n">
-        <x:v>0.1024688080700823</x:v>
-      </x:c>
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="T47"/>
       <x:c r="U47"/>
     </x:row>
     <x:row r="48">
@@ -27710,24 +27706,24 @@
         <x:v>561</x:v>
       </x:c>
       <x:c r="E48" t="n">
-        <x:v>283.6477987421384</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="F48" t="n">
-        <x:v>346.54088050314465</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="G48"/>
       <x:c r="H48"/>
       <x:c r="I48" t="n">
-        <x:v>45.874213836477985</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J48" t="n">
-        <x:v>74.88469601677149</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="K48" t="n">
-        <x:v>825.3249475890985</x:v>
+        <x:v>959</x:v>
       </x:c>
       <x:c r="L48" t="n">
-        <x:v>213836.4779874214</x:v>
+        <x:v>226282</x:v>
       </x:c>
       <x:c r="M48"/>
       <x:c r="N48"/>
@@ -27736,11 +27732,9 @@
       <x:c r="Q48"/>
       <x:c r="R48"/>
       <x:c r="S48" t="n">
-        <x:v>255.59748427672955</x:v>
-      </x:c>
-      <x:c r="T48" t="n">
-        <x:v>0.10985324947589098</x:v>
-      </x:c>
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="T48"/>
       <x:c r="U48"/>
     </x:row>
   </x:sheetData>

</xml_diff>